<commit_message>
Update spider results 2026-08-14 03:27:03
</commit_message>
<xml_diff>
--- a/current.xlsx
+++ b/current.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F538"/>
+  <dimension ref="A1:F539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17632,6 +17632,38 @@
         </is>
       </c>
     </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>上海市</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>松江区</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>松江区</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>沪亭北路邮政所</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>信件、印刷品、包裹、邮政汇兑、国际业务、港澳台业务、报刊订阅</t>
+        </is>
+      </c>
+      <c r="F539" t="inlineStr">
+        <is>
+          <t>https://zwfw.spb.gov.cn/sj/310000/pfyycsml/pfyycsmlDetail?uuid=56826</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>